<commit_message>
add: location, building, loss_payee data loading and mapping
</commit_message>
<xml_diff>
--- a/src/data/output/apd_cargo_combined_output.xlsx
+++ b/src/data/output/apd_cargo_combined_output.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{746828EE-F2A7-42A2-B9C1-CCF450798ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Output" state="visible" r:id="rId4"/>
+    <sheet name="Output" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="357">
   <si>
     <t>Test ID</t>
   </si>
@@ -827,32 +831,287 @@
   </si>
   <si>
     <t>TS-080</t>
+  </si>
+  <si>
+    <t>0098690</t>
+  </si>
+  <si>
+    <t>13896.00</t>
+  </si>
+  <si>
+    <t>1210.00</t>
+  </si>
+  <si>
+    <t>687.32</t>
+  </si>
+  <si>
+    <t>15793.32</t>
+  </si>
+  <si>
+    <t>0098695</t>
+  </si>
+  <si>
+    <t>11423.00</t>
+  </si>
+  <si>
+    <t>150.00</t>
+  </si>
+  <si>
+    <t>231.46</t>
+  </si>
+  <si>
+    <t>11804.46</t>
+  </si>
+  <si>
+    <t>0098688</t>
+  </si>
+  <si>
+    <t>6682.00</t>
+  </si>
+  <si>
+    <t>200.46</t>
+  </si>
+  <si>
+    <t>7382.46</t>
+  </si>
+  <si>
+    <t>0098692</t>
+  </si>
+  <si>
+    <t>3846.00</t>
+  </si>
+  <si>
+    <t>555.00</t>
+  </si>
+  <si>
+    <t>115.38</t>
+  </si>
+  <si>
+    <t>4516.38</t>
+  </si>
+  <si>
+    <t>0098691</t>
+  </si>
+  <si>
+    <t>6569.00</t>
+  </si>
+  <si>
+    <t>475.00</t>
+  </si>
+  <si>
+    <t>140.88</t>
+  </si>
+  <si>
+    <t>7184.88</t>
+  </si>
+  <si>
+    <t>0098693</t>
+  </si>
+  <si>
+    <t>5972.00</t>
+  </si>
+  <si>
+    <t>179.16</t>
+  </si>
+  <si>
+    <t>6651.16</t>
+  </si>
+  <si>
+    <t>0098689</t>
+  </si>
+  <si>
+    <t>18059.00</t>
+  </si>
+  <si>
+    <t>650.00</t>
+  </si>
+  <si>
+    <t>851.26</t>
+  </si>
+  <si>
+    <t>19560.26</t>
+  </si>
+  <si>
+    <t>0098694</t>
+  </si>
+  <si>
+    <t>18803.00</t>
+  </si>
+  <si>
+    <t>181.41</t>
+  </si>
+  <si>
+    <t>940.15</t>
+  </si>
+  <si>
+    <t>19924.56</t>
+  </si>
+  <si>
+    <t>0098701</t>
+  </si>
+  <si>
+    <t>10114.00</t>
+  </si>
+  <si>
+    <t>1015.34</t>
+  </si>
+  <si>
+    <t>505.70</t>
+  </si>
+  <si>
+    <t>11635.04</t>
+  </si>
+  <si>
+    <t>0098700</t>
+  </si>
+  <si>
+    <t>7639.00</t>
+  </si>
+  <si>
+    <t>545.00</t>
+  </si>
+  <si>
+    <t>372.37</t>
+  </si>
+  <si>
+    <t>8556.37</t>
+  </si>
+  <si>
+    <t>0098702</t>
+  </si>
+  <si>
+    <t>10373.00</t>
+  </si>
+  <si>
+    <t>666.12</t>
+  </si>
+  <si>
+    <t>518.65</t>
+  </si>
+  <si>
+    <t>11557.77</t>
+  </si>
+  <si>
+    <t>0098704</t>
+  </si>
+  <si>
+    <t>14117.00</t>
+  </si>
+  <si>
+    <t>235.00</t>
+  </si>
+  <si>
+    <t>653.02</t>
+  </si>
+  <si>
+    <t>15005.02</t>
+  </si>
+  <si>
+    <t>0098714</t>
+  </si>
+  <si>
+    <t>9121.00</t>
+  </si>
+  <si>
+    <t>167.36</t>
+  </si>
+  <si>
+    <t>456.05</t>
+  </si>
+  <si>
+    <t>9744.41</t>
+  </si>
+  <si>
+    <t>0098718</t>
+  </si>
+  <si>
+    <t>6586.00</t>
+  </si>
+  <si>
+    <t>824.76</t>
+  </si>
+  <si>
+    <t>329.30</t>
+  </si>
+  <si>
+    <t>7740.06</t>
+  </si>
+  <si>
+    <t>0098720</t>
+  </si>
+  <si>
+    <t>6018.00</t>
+  </si>
+  <si>
+    <t>640.00</t>
+  </si>
+  <si>
+    <t>199.74</t>
+  </si>
+  <si>
+    <t>6857.74</t>
+  </si>
+  <si>
+    <t>0098719</t>
+  </si>
+  <si>
+    <t>6542.00</t>
+  </si>
+  <si>
+    <t>164.52</t>
+  </si>
+  <si>
+    <t>7479.08</t>
+  </si>
+  <si>
+    <t>0098729</t>
+  </si>
+  <si>
+    <t>6719.00</t>
+  </si>
+  <si>
+    <t>201.57</t>
+  </si>
+  <si>
+    <t>7195.57</t>
+  </si>
+  <si>
+    <t>0098730</t>
+  </si>
+  <si>
+    <t>9984.00</t>
+  </si>
+  <si>
+    <t>235.32</t>
+  </si>
+  <si>
+    <t>10697.98</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
       <color rgb="FF2C3E50"/>
-      <sz val="12"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF000000"/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -884,10 +1143,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1226,23 +1483,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I121"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.571428571428571" customWidth="1"/>
-    <col min="2" max="2" width="13.857142857142858" customWidth="1"/>
-    <col min="3" max="3" width="15.142857142857142" customWidth="1"/>
-    <col min="4" max="4" width="13.857142857142858" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="13.571428571428571" customWidth="1"/>
-    <col min="7" max="7" width="18.857142857142858" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" customWidth="1"/>
+    <col min="7" max="7" width="18.88671875" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="25.428571428571427" customWidth="1"/>
-    <col min="10" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="9" max="9" width="25.44140625" customWidth="1"/>
+    <col min="10" max="24" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1271,1743 +1528,1923 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="12.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>1739.76</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="4">
         <v>61866.76</v>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="12.6" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="4">
         <v>972.75</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="4">
         <v>22351.75</v>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="12.6" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="4">
         <v>307.94</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="4">
         <v>7075.94</v>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="12.6" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="4">
         <v>440.61</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="4">
         <v>15797.61</v>
       </c>
     </row>
-    <row r="6" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="12.6" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="3">
-        <v>18083.99</v>
-      </c>
-    </row>
-    <row r="7" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F6" s="4">
+        <v>18083.990000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="12.6" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="4">
         <v>162.16</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="4">
         <v>7371.68</v>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="12.6" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="4">
         <v>1691.58</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="4">
         <v>1526.35</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="4">
         <v>33744.93</v>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="12.6" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="4">
         <v>444.26</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="4">
         <v>22657.26</v>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="12.6" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="3">
-        <v>566.57</v>
-      </c>
-      <c r="F10" s="3">
+      <c r="E10" s="4">
+        <v>566.57000000000005</v>
+      </c>
+      <c r="F10" s="4">
         <v>13018.57</v>
       </c>
     </row>
-    <row r="11" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="12.6" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="12.6" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="4">
         <v>6114.59</v>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="12.6" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="12.6" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="4">
         <v>456.65</v>
       </c>
-      <c r="F14" s="3">
-        <v>10167.05</v>
-      </c>
-    </row>
-    <row r="15" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F14" s="4">
+        <v>10167.049999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="12.6" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="4">
         <v>177.54</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="4">
         <v>6865.54</v>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="12.6" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-    </row>
-    <row r="17" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="12.6" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="4">
         <v>404.04</v>
       </c>
-      <c r="F17" s="3">
-        <v>9284.04</v>
-      </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F17" s="4">
+        <v>9284.0400000000009</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="12.6" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="4">
         <v>184.02</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="4">
         <v>6658.02</v>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="12.6" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="3">
+      <c r="E19" s="4">
         <v>461.24</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="4">
         <v>10598.24</v>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="12.6" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E20" s="4">
         <v>117.15</v>
       </c>
-      <c r="F20" s="3">
-        <v>4252.15</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F20" s="4">
+        <v>4252.1499999999996</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="12.6" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="4">
         <v>972.13</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21" s="4">
         <v>618.85</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="4">
         <v>13967.98</v>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="12.6" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D22" s="3">
-        <v>264.03</v>
-      </c>
-      <c r="E22" s="3">
+      <c r="D22" s="4">
+        <v>264.02999999999997</v>
+      </c>
+      <c r="E22" s="4">
         <v>233.85</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="4">
         <v>5174.88</v>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="12.6" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="4">
         <v>599.41</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F23" s="4">
         <v>10893.61</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="12.6" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="12.6" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25" s="4">
         <v>373.19</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F25" s="4">
         <v>4991.09</v>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="12.6" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26" s="4">
         <v>281.64</v>
       </c>
-      <c r="F26" s="3">
+      <c r="F26" s="4">
         <v>6471.64</v>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="12.6" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27" s="4">
         <v>901.68</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E27" s="4">
         <v>611.35</v>
       </c>
-      <c r="F27" s="3">
+      <c r="F27" s="4">
         <v>13740.03</v>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="12.6" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28" s="4">
         <v>325.02</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28" s="4">
         <v>11449.02</v>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="12.6" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E29" s="4">
         <v>169.94</v>
       </c>
-      <c r="F29" s="3">
+      <c r="F29" s="4">
         <v>3904.94</v>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="12.6" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E30" s="4">
         <v>280.89</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="4">
         <v>9643.89</v>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="12.6" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="E31" s="3">
+      <c r="E31" s="4">
         <v>169.77</v>
       </c>
-      <c r="F31" s="3">
+      <c r="F31" s="4">
         <v>6103.77</v>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="12.6" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="E32" s="3">
+      <c r="E32" s="4">
         <v>424.83</v>
       </c>
-      <c r="F32" s="3">
+      <c r="F32" s="4">
         <v>14585.83</v>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="12.6" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E33" s="3">
+      <c r="E33" s="4">
         <v>157.26</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F33" s="4">
         <v>8020.26</v>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="12.6" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="D34" s="3">
-        <v>545.07</v>
-      </c>
-      <c r="E34" s="3" t="s">
+      <c r="D34" s="4">
+        <v>545.07000000000005</v>
+      </c>
+      <c r="E34" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="F34" s="3">
+      <c r="F34" s="4">
         <v>5818.17</v>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="12.6" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="E35" s="3">
+      <c r="E35" s="4">
         <v>189.84</v>
       </c>
-      <c r="F35" s="3">
+      <c r="F35" s="4">
         <v>9681.84</v>
       </c>
     </row>
-    <row r="36" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="12.6" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36" s="4">
         <v>537.88</v>
       </c>
-      <c r="E36" s="3">
+      <c r="E36" s="4">
         <v>464.65</v>
       </c>
-      <c r="F36" s="3">
-        <v>10295.53</v>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F36" s="4">
+        <v>10295.530000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="12.6" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="E37" s="3">
+      <c r="E37" s="4">
         <v>164.19</v>
       </c>
-      <c r="F37" s="3">
+      <c r="F37" s="4">
         <v>6292.19</v>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="12.6" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="E38" s="3">
+      <c r="E38" s="4">
         <v>194.61</v>
       </c>
-      <c r="F38" s="3">
+      <c r="F38" s="4">
         <v>6681.61</v>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="12.6" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
-    </row>
-    <row r="40" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B39" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="12.6" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="E40" s="3">
+      <c r="E40" s="4">
         <v>218.37</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40" s="4">
         <v>7497.37</v>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="12.6" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
-      <c r="F41" s="3"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B41" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="12.6" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
-    </row>
-    <row r="43" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B42" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="12.6" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="E43" s="3">
+      <c r="E43" s="4">
         <v>168.93</v>
       </c>
-      <c r="F43" s="3">
+      <c r="F43" s="4">
         <v>7679.56</v>
       </c>
     </row>
-    <row r="44" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="12.6" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="E44" s="3">
+      <c r="E44" s="4">
         <v>428.49</v>
       </c>
-      <c r="F44" s="3">
+      <c r="F44" s="4">
         <v>14711.49</v>
       </c>
     </row>
-    <row r="45" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" ht="12.6" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-      <c r="F45" s="3"/>
-    </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B45" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="12.6" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="E46" s="3">
+      <c r="E46" s="4">
         <v>130.26</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F46" s="4">
         <v>4722.26</v>
       </c>
     </row>
-    <row r="47" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" ht="12.6" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="D47" s="3" t="s">
+      <c r="D47" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="E47" s="3">
+      <c r="E47" s="4">
         <v>264.33</v>
       </c>
-      <c r="F47" s="3">
+      <c r="F47" s="4">
         <v>9075.33</v>
       </c>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="12.6" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
-    </row>
-    <row r="49" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B48" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="12.6" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="B49" s="3" t="s">
+      <c r="B49" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C49" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="D49" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="E49" s="3">
-        <v>258.78</v>
-      </c>
-      <c r="F49" s="3">
-        <v>9784.78</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E49" s="4">
+        <v>258.77999999999997</v>
+      </c>
+      <c r="F49" s="4">
+        <v>9784.7800000000007</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="12.6" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="C50" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="D50" s="3" t="s">
+      <c r="D50" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="E50" s="3">
+      <c r="E50" s="4">
         <v>248.56</v>
       </c>
-      <c r="F50" s="3">
+      <c r="F50" s="4">
         <v>5711.56</v>
       </c>
     </row>
-    <row r="51" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="12.6" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="B51" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C51" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="D51" s="3">
+      <c r="D51" s="4">
         <v>1259.23</v>
       </c>
-      <c r="E51" s="3">
-        <v>539.67</v>
-      </c>
-      <c r="F51" s="3" t="s">
+      <c r="E51" s="4">
+        <v>539.66999999999996</v>
+      </c>
+      <c r="F51" s="4" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="12.6" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-    </row>
-    <row r="53" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B52" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="12.6" customHeight="1">
       <c r="A53" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B53" s="3" t="s">
+      <c r="B53" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C53" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="D53" s="3" t="s">
+      <c r="D53" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="E53" s="3">
-        <v>155.73</v>
-      </c>
-      <c r="F53" s="3">
+      <c r="E53" s="4">
+        <v>155.72999999999999</v>
+      </c>
+      <c r="F53" s="4">
         <v>5346.73</v>
       </c>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="12.6" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="B54" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="D54" s="3">
+      <c r="D54" s="4">
         <v>435.57</v>
       </c>
-      <c r="E54" s="3" t="s">
+      <c r="E54" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="F54" s="3">
+      <c r="F54" s="4">
         <v>7636.47</v>
       </c>
     </row>
-    <row r="55" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" ht="12.6" customHeight="1">
       <c r="A55" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="D55" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="E55" s="3">
+      <c r="E55" s="4">
         <v>138.51</v>
       </c>
-      <c r="F55" s="3">
+      <c r="F55" s="4">
         <v>6296.66</v>
       </c>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="12.6" customHeight="1">
       <c r="A56" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
-      <c r="E56" s="3"/>
-      <c r="F56" s="3"/>
-    </row>
-    <row r="57" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B56" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="12.6" customHeight="1">
       <c r="A57" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="B57" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C57" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="D57" s="3" t="s">
+      <c r="D57" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="E57" s="3">
+      <c r="E57" s="4">
         <v>194.44</v>
       </c>
-      <c r="F57" s="3">
+      <c r="F57" s="4">
         <v>9916.44</v>
       </c>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" ht="12.6" customHeight="1">
       <c r="A58" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-    </row>
-    <row r="59" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B58" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="12.6" customHeight="1">
       <c r="A59" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="B59" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="C59" s="3" t="s">
+      <c r="C59" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="D59" s="3">
+      <c r="D59" s="4">
         <v>893.72</v>
       </c>
-      <c r="E59" s="3">
+      <c r="E59" s="4">
         <v>395.25</v>
       </c>
-      <c r="F59" s="3">
-        <v>9193.97</v>
-      </c>
-    </row>
-    <row r="60" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F59" s="4">
+        <v>9193.9699999999993</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="12.6" customHeight="1">
       <c r="A60" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="B60" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="C60" s="3" t="s">
+      <c r="C60" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="D60" s="3">
+      <c r="D60" s="4">
         <v>203.25</v>
       </c>
-      <c r="E60" s="3" t="s">
+      <c r="E60" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="F60" s="3">
+      <c r="F60" s="4">
         <v>15342.15</v>
       </c>
     </row>
-    <row r="61" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" ht="12.6" customHeight="1">
       <c r="A61" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B61" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="C61" s="3" t="s">
+      <c r="C61" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="D61" s="3" t="s">
+      <c r="D61" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="E61" s="3">
+      <c r="E61" s="4">
         <v>172.35</v>
       </c>
-      <c r="F61" s="3">
+      <c r="F61" s="4">
         <v>6252.35</v>
       </c>
     </row>
-    <row r="62" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" ht="12.6" customHeight="1">
       <c r="A62" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="B62" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="D62" s="3" t="s">
+      <c r="D62" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="E62" s="3">
+      <c r="E62" s="4">
         <v>494.91</v>
       </c>
-      <c r="F62" s="3">
+      <c r="F62" s="4">
         <v>11371.91</v>
       </c>
     </row>
-    <row r="63" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" ht="12.6" customHeight="1">
       <c r="A63" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="3"/>
-      <c r="E63" s="3"/>
-      <c r="F63" s="3"/>
-    </row>
-    <row r="64" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B63" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="12.6" customHeight="1">
       <c r="A64" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
-      <c r="E64" s="3"/>
-      <c r="F64" s="3"/>
-    </row>
-    <row r="65" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B64" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="12.6" customHeight="1">
       <c r="A65" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B65" s="3" t="s">
+      <c r="B65" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="D65" s="3" t="s">
+      <c r="D65" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="E65" s="3">
+      <c r="E65" s="4">
         <v>363.32</v>
       </c>
-      <c r="F65" s="3">
+      <c r="F65" s="4">
         <v>8348.32</v>
       </c>
     </row>
-    <row r="66" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="12.6" customHeight="1">
       <c r="A66" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="B66" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C66" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="D66" s="3" t="s">
+      <c r="D66" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="E66" s="3">
+      <c r="E66" s="4">
         <v>162.06</v>
       </c>
-      <c r="F66" s="3">
+      <c r="F66" s="4">
         <v>6064.06</v>
       </c>
     </row>
-    <row r="67" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" ht="12.6" customHeight="1">
       <c r="A67" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="B67" s="3" t="s">
+      <c r="B67" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C67" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="D67" s="3" t="s">
+      <c r="D67" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="E67" s="3">
+      <c r="E67" s="4">
         <v>197.25</v>
       </c>
-      <c r="F67" s="3">
+      <c r="F67" s="4">
         <v>8967.32</v>
       </c>
     </row>
-    <row r="68" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" ht="12.6" customHeight="1">
       <c r="A68" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
-    </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B68" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="12.6" customHeight="1">
       <c r="A69" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="B69" s="3" t="s">
+      <c r="B69" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="C69" s="3" t="s">
+      <c r="C69" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="D69" s="3" t="s">
+      <c r="D69" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="E69" s="3">
+      <c r="E69" s="4">
         <v>188.58</v>
       </c>
-      <c r="F69" s="3">
+      <c r="F69" s="4">
         <v>7214.58</v>
       </c>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="12.6" customHeight="1">
       <c r="A70" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="B70" s="3" t="s">
+      <c r="B70" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="D70" s="3" t="s">
+      <c r="D70" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="E70" s="3" t="s">
+      <c r="E70" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="F70" s="3" t="s">
+      <c r="F70" s="4" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="71" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" ht="12.6" customHeight="1">
       <c r="A71" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B71" s="3" t="s">
+      <c r="B71" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C71" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="D71" s="3" t="s">
+      <c r="D71" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="E71" s="3">
+      <c r="E71" s="4">
         <v>442.14</v>
       </c>
-      <c r="F71" s="3">
+      <c r="F71" s="4">
         <v>15180.14</v>
       </c>
     </row>
-    <row r="72" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" ht="12.6" customHeight="1">
       <c r="A72" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="B72" s="3" t="s">
+      <c r="B72" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C72" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="D72" s="3" t="s">
+      <c r="D72" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E72" s="3">
+      <c r="E72" s="4">
         <v>218.08</v>
       </c>
-      <c r="F72" s="3">
+      <c r="F72" s="4">
         <v>5011.08</v>
       </c>
     </row>
-    <row r="73" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="12.6" customHeight="1">
       <c r="A73" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-    </row>
-    <row r="74" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B73" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="12.6" customHeight="1">
       <c r="A74" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="B74" s="3" t="s">
+      <c r="B74" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="C74" s="3" t="s">
+      <c r="C74" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="D74" s="3" t="s">
+      <c r="D74" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="E74" s="3">
+      <c r="E74" s="4">
         <v>352.44</v>
       </c>
-      <c r="F74" s="3">
+      <c r="F74" s="4">
         <v>12100.44</v>
       </c>
     </row>
-    <row r="75" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" ht="12.6" customHeight="1">
       <c r="A75" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="B75" s="3" t="s">
+      <c r="B75" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="C75" s="3" t="s">
+      <c r="C75" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="D75" s="3" t="s">
+      <c r="D75" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E75" s="3">
+      <c r="E75" s="4">
         <v>146.47</v>
       </c>
-      <c r="F75" s="3">
+      <c r="F75" s="4">
         <v>6658.75</v>
       </c>
     </row>
-    <row r="76" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" ht="12.6" customHeight="1">
       <c r="A76" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B76" s="3"/>
-      <c r="C76" s="3"/>
-      <c r="D76" s="3"/>
-      <c r="E76" s="3"/>
-      <c r="F76" s="3"/>
-    </row>
-    <row r="77" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B76" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="12.6" customHeight="1">
       <c r="A77" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="B77" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="C77" s="3" t="s">
+      <c r="C77" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="D77" s="3" t="s">
+      <c r="D77" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="E77" s="3">
+      <c r="E77" s="4">
         <v>214.77</v>
       </c>
-      <c r="F77" s="3">
+      <c r="F77" s="4">
         <v>7373.77</v>
       </c>
     </row>
-    <row r="78" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" ht="12.6" customHeight="1">
       <c r="A78" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="B78" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C78" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="D78" s="3" t="s">
+      <c r="D78" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="E78" s="3">
+      <c r="E78" s="4">
         <v>245.37</v>
       </c>
-      <c r="F78" s="3">
+      <c r="F78" s="4">
         <v>11154.19</v>
       </c>
     </row>
-    <row r="79" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" ht="12.6" customHeight="1">
       <c r="A79" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="B79" s="3"/>
-      <c r="C79" s="3"/>
-      <c r="D79" s="3"/>
-      <c r="E79" s="3"/>
-      <c r="F79" s="3"/>
-    </row>
-    <row r="80" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B79" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="12.6" customHeight="1">
       <c r="A80" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="B80" s="3"/>
-      <c r="C80" s="3"/>
-      <c r="D80" s="3"/>
-      <c r="E80" s="3"/>
-      <c r="F80" s="3"/>
-    </row>
-    <row r="81" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B80" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="E80" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="12.6" customHeight="1">
       <c r="A81" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B81" s="3"/>
-      <c r="C81" s="3"/>
-      <c r="D81" s="3"/>
-      <c r="E81" s="3"/>
-      <c r="F81" s="3"/>
-    </row>
-    <row r="82" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B81" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="E81" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="12.6" customHeight="1">
       <c r="A82" s="2"/>
-      <c r="B82" s="4"/>
-      <c r="C82" s="4"/>
-      <c r="D82" s="4"/>
-      <c r="E82" s="4"/>
-      <c r="F82" s="4"/>
-    </row>
-    <row r="83" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B82" s="3"/>
+      <c r="C82" s="3"/>
+      <c r="D82" s="3"/>
+      <c r="E82" s="3"/>
+      <c r="F82" s="3"/>
+    </row>
+    <row r="83" spans="1:6" ht="12.6" customHeight="1">
       <c r="A83" s="2"/>
-      <c r="B83" s="4"/>
-      <c r="C83" s="4"/>
-      <c r="D83" s="4"/>
-      <c r="E83" s="4"/>
-      <c r="F83" s="4"/>
-    </row>
-    <row r="84" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B83" s="3"/>
+      <c r="C83" s="3"/>
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
+    </row>
+    <row r="84" spans="1:6" ht="12.6" customHeight="1">
       <c r="A84" s="2"/>
-      <c r="B84" s="4"/>
-      <c r="C84" s="4"/>
-      <c r="D84" s="4"/>
-      <c r="E84" s="4"/>
-      <c r="F84" s="4"/>
-    </row>
-    <row r="85" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B84" s="3"/>
+      <c r="C84" s="3"/>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+    </row>
+    <row r="85" spans="1:6" ht="12.6" customHeight="1">
       <c r="A85" s="2"/>
-      <c r="B85" s="4"/>
-      <c r="C85" s="4"/>
-      <c r="D85" s="4"/>
-      <c r="E85" s="4"/>
-      <c r="F85" s="4"/>
-    </row>
-    <row r="86" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B85" s="3"/>
+      <c r="C85" s="3"/>
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
+    </row>
+    <row r="86" spans="1:6" ht="12.6" customHeight="1">
       <c r="A86" s="2"/>
-      <c r="B86" s="4"/>
-      <c r="C86" s="4"/>
-      <c r="D86" s="4"/>
-      <c r="E86" s="4"/>
-      <c r="F86" s="4"/>
-    </row>
-    <row r="87" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B86" s="3"/>
+      <c r="C86" s="3"/>
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3"/>
+    </row>
+    <row r="87" spans="1:6" ht="12.6" customHeight="1">
       <c r="A87" s="2"/>
-      <c r="B87" s="4"/>
-      <c r="C87" s="4"/>
-      <c r="D87" s="4"/>
-      <c r="E87" s="4"/>
-      <c r="F87" s="4"/>
-    </row>
-    <row r="88" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B87" s="3"/>
+      <c r="C87" s="3"/>
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+    </row>
+    <row r="88" spans="1:6" ht="12.6" customHeight="1">
       <c r="A88" s="2"/>
-      <c r="B88" s="4"/>
-      <c r="C88" s="4"/>
-      <c r="D88" s="4"/>
-      <c r="E88" s="4"/>
-      <c r="F88" s="4"/>
-    </row>
-    <row r="89" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B88" s="3"/>
+      <c r="C88" s="3"/>
+      <c r="D88" s="3"/>
+      <c r="E88" s="3"/>
+      <c r="F88" s="3"/>
+    </row>
+    <row r="89" spans="1:6" ht="12.6" customHeight="1">
       <c r="A89" s="2"/>
-      <c r="B89" s="4"/>
-      <c r="C89" s="4"/>
-      <c r="D89" s="4"/>
-      <c r="E89" s="4"/>
-      <c r="F89" s="4"/>
-    </row>
-    <row r="90" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B89" s="3"/>
+      <c r="C89" s="3"/>
+      <c r="D89" s="3"/>
+      <c r="E89" s="3"/>
+      <c r="F89" s="3"/>
+    </row>
+    <row r="90" spans="1:6" ht="12.6" customHeight="1">
       <c r="A90" s="2"/>
-      <c r="B90" s="4"/>
-      <c r="C90" s="4"/>
-      <c r="D90" s="4"/>
-      <c r="E90" s="4"/>
-      <c r="F90" s="4"/>
-    </row>
-    <row r="91" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B90" s="3"/>
+      <c r="C90" s="3"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3"/>
+    </row>
+    <row r="91" spans="1:6" ht="12.6" customHeight="1">
       <c r="A91" s="2"/>
-      <c r="B91" s="4"/>
-      <c r="C91" s="4"/>
-      <c r="D91" s="4"/>
-      <c r="E91" s="4"/>
-      <c r="F91" s="4"/>
-    </row>
-    <row r="92" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B91" s="3"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="3"/>
+      <c r="E91" s="3"/>
+      <c r="F91" s="3"/>
+    </row>
+    <row r="92" spans="1:6" ht="12.6" customHeight="1">
       <c r="A92" s="2"/>
-      <c r="B92" s="4"/>
-      <c r="C92" s="4"/>
-      <c r="D92" s="4"/>
-      <c r="E92" s="4"/>
-      <c r="F92" s="4"/>
-    </row>
-    <row r="93" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B92" s="3"/>
+      <c r="C92" s="3"/>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+    </row>
+    <row r="93" spans="1:6" ht="12.6" customHeight="1">
       <c r="A93" s="2"/>
-      <c r="B93" s="4"/>
-      <c r="C93" s="4"/>
-      <c r="D93" s="4"/>
-      <c r="E93" s="4"/>
-      <c r="F93" s="4"/>
-    </row>
-    <row r="94" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B93" s="3"/>
+      <c r="C93" s="3"/>
+      <c r="D93" s="3"/>
+      <c r="E93" s="3"/>
+      <c r="F93" s="3"/>
+    </row>
+    <row r="94" spans="1:6" ht="12.6" customHeight="1">
       <c r="A94" s="2"/>
-      <c r="B94" s="4"/>
-      <c r="C94" s="4"/>
-      <c r="D94" s="4"/>
-      <c r="E94" s="4"/>
-      <c r="F94" s="4"/>
-    </row>
-    <row r="95" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B94" s="3"/>
+      <c r="C94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+    </row>
+    <row r="95" spans="1:6" ht="12.6" customHeight="1">
       <c r="A95" s="2"/>
-      <c r="B95" s="4"/>
-      <c r="C95" s="4"/>
-      <c r="D95" s="4"/>
-      <c r="E95" s="4"/>
-      <c r="F95" s="4"/>
-    </row>
-    <row r="96" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B95" s="3"/>
+      <c r="C95" s="3"/>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+      <c r="F95" s="3"/>
+    </row>
+    <row r="96" spans="1:6" ht="12.6" customHeight="1">
       <c r="A96" s="2"/>
-      <c r="B96" s="4"/>
-      <c r="C96" s="4"/>
-      <c r="D96" s="4"/>
-      <c r="E96" s="4"/>
-      <c r="F96" s="4"/>
-    </row>
-    <row r="97" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B96" s="3"/>
+      <c r="C96" s="3"/>
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+      <c r="F96" s="3"/>
+    </row>
+    <row r="97" spans="1:6" ht="12.6" customHeight="1">
       <c r="A97" s="2"/>
-      <c r="B97" s="4"/>
-      <c r="C97" s="4"/>
-      <c r="D97" s="4"/>
-      <c r="E97" s="4"/>
-      <c r="F97" s="4"/>
-    </row>
-    <row r="98" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B97" s="3"/>
+      <c r="C97" s="3"/>
+      <c r="D97" s="3"/>
+      <c r="E97" s="3"/>
+      <c r="F97" s="3"/>
+    </row>
+    <row r="98" spans="1:6" ht="12.6" customHeight="1">
       <c r="A98" s="2"/>
-      <c r="B98" s="4"/>
-      <c r="C98" s="4"/>
-      <c r="D98" s="4"/>
-      <c r="E98" s="4"/>
-      <c r="F98" s="4"/>
-    </row>
-    <row r="99" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B98" s="3"/>
+      <c r="C98" s="3"/>
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+    </row>
+    <row r="99" spans="1:6" ht="12.6" customHeight="1">
       <c r="A99" s="2"/>
-      <c r="B99" s="4"/>
-      <c r="C99" s="4"/>
-      <c r="D99" s="4"/>
-      <c r="E99" s="4"/>
-      <c r="F99" s="4"/>
-    </row>
-    <row r="100" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B99" s="3"/>
+      <c r="C99" s="3"/>
+      <c r="D99" s="3"/>
+      <c r="E99" s="3"/>
+      <c r="F99" s="3"/>
+    </row>
+    <row r="100" spans="1:6" ht="12.6" customHeight="1">
       <c r="A100" s="2"/>
-      <c r="B100" s="4"/>
-      <c r="C100" s="4"/>
-      <c r="D100" s="4"/>
-      <c r="E100" s="4"/>
-      <c r="F100" s="4"/>
-    </row>
-    <row r="101" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B100" s="3"/>
+      <c r="C100" s="3"/>
+      <c r="D100" s="3"/>
+      <c r="E100" s="3"/>
+      <c r="F100" s="3"/>
+    </row>
+    <row r="101" spans="1:6" ht="12.6" customHeight="1">
       <c r="A101" s="2"/>
-      <c r="B101" s="4"/>
-      <c r="C101" s="4"/>
-      <c r="D101" s="4"/>
-      <c r="E101" s="4"/>
-      <c r="F101" s="4"/>
-    </row>
-    <row r="102" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B101" s="3"/>
+      <c r="C101" s="3"/>
+      <c r="D101" s="3"/>
+      <c r="E101" s="3"/>
+      <c r="F101" s="3"/>
+    </row>
+    <row r="102" spans="1:6" ht="12.6" customHeight="1">
       <c r="A102" s="2"/>
-      <c r="B102" s="4"/>
-      <c r="C102" s="4"/>
-      <c r="D102" s="4"/>
-      <c r="E102" s="4"/>
-      <c r="F102" s="4"/>
-    </row>
-    <row r="103" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B102" s="3"/>
+      <c r="C102" s="3"/>
+      <c r="D102" s="3"/>
+      <c r="E102" s="3"/>
+      <c r="F102" s="3"/>
+    </row>
+    <row r="103" spans="1:6" ht="12.6" customHeight="1">
       <c r="A103" s="2"/>
-      <c r="B103" s="4"/>
-      <c r="C103" s="4"/>
-      <c r="D103" s="4"/>
-      <c r="E103" s="4"/>
-      <c r="F103" s="4"/>
-    </row>
-    <row r="104" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B103" s="3"/>
+      <c r="C103" s="3"/>
+      <c r="D103" s="3"/>
+      <c r="E103" s="3"/>
+      <c r="F103" s="3"/>
+    </row>
+    <row r="104" spans="1:6" ht="12.6" customHeight="1">
       <c r="A104" s="2"/>
-      <c r="B104" s="4"/>
-      <c r="C104" s="4"/>
-      <c r="D104" s="4"/>
-      <c r="E104" s="4"/>
-      <c r="F104" s="4"/>
-    </row>
-    <row r="105" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B104" s="3"/>
+      <c r="C104" s="3"/>
+      <c r="D104" s="3"/>
+      <c r="E104" s="3"/>
+      <c r="F104" s="3"/>
+    </row>
+    <row r="105" spans="1:6" ht="12.6" customHeight="1">
       <c r="A105" s="2"/>
-      <c r="B105" s="4"/>
-      <c r="C105" s="4"/>
-      <c r="D105" s="4"/>
-      <c r="E105" s="4"/>
-      <c r="F105" s="4"/>
-    </row>
-    <row r="106" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B105" s="3"/>
+      <c r="C105" s="3"/>
+      <c r="D105" s="3"/>
+      <c r="E105" s="3"/>
+      <c r="F105" s="3"/>
+    </row>
+    <row r="106" spans="1:6" ht="12.6" customHeight="1">
       <c r="A106" s="2"/>
-      <c r="B106" s="4"/>
-      <c r="C106" s="4"/>
-      <c r="D106" s="4"/>
-      <c r="E106" s="4"/>
-      <c r="F106" s="4"/>
-    </row>
-    <row r="107" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B106" s="3"/>
+      <c r="C106" s="3"/>
+      <c r="D106" s="3"/>
+      <c r="E106" s="3"/>
+      <c r="F106" s="3"/>
+    </row>
+    <row r="107" spans="1:6" ht="12.6" customHeight="1">
       <c r="A107" s="2"/>
-      <c r="B107" s="4"/>
-      <c r="C107" s="4"/>
-      <c r="D107" s="4"/>
-      <c r="E107" s="4"/>
-      <c r="F107" s="4"/>
-    </row>
-    <row r="108" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B107" s="3"/>
+      <c r="C107" s="3"/>
+      <c r="D107" s="3"/>
+      <c r="E107" s="3"/>
+      <c r="F107" s="3"/>
+    </row>
+    <row r="108" spans="1:6" ht="12.6" customHeight="1">
       <c r="A108" s="2"/>
-      <c r="B108" s="4"/>
-      <c r="C108" s="4"/>
-      <c r="D108" s="4"/>
-      <c r="E108" s="4"/>
-      <c r="F108" s="4"/>
-    </row>
-    <row r="109" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B108" s="3"/>
+      <c r="C108" s="3"/>
+      <c r="D108" s="3"/>
+      <c r="E108" s="3"/>
+      <c r="F108" s="3"/>
+    </row>
+    <row r="109" spans="1:6" ht="12.6" customHeight="1">
       <c r="A109" s="2"/>
-      <c r="B109" s="4"/>
-      <c r="C109" s="4"/>
-      <c r="D109" s="4"/>
-      <c r="E109" s="4"/>
-      <c r="F109" s="4"/>
-    </row>
-    <row r="110" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B109" s="3"/>
+      <c r="C109" s="3"/>
+      <c r="D109" s="3"/>
+      <c r="E109" s="3"/>
+      <c r="F109" s="3"/>
+    </row>
+    <row r="110" spans="1:6" ht="12.6" customHeight="1">
       <c r="A110" s="2"/>
-      <c r="B110" s="4"/>
-      <c r="C110" s="4"/>
-      <c r="D110" s="4"/>
-      <c r="E110" s="4"/>
-      <c r="F110" s="4"/>
-    </row>
-    <row r="111" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B110" s="3"/>
+      <c r="C110" s="3"/>
+      <c r="D110" s="3"/>
+      <c r="E110" s="3"/>
+      <c r="F110" s="3"/>
+    </row>
+    <row r="111" spans="1:6" ht="12.6" customHeight="1">
       <c r="A111" s="2"/>
-      <c r="B111" s="4"/>
-      <c r="C111" s="4"/>
-      <c r="D111" s="4"/>
-      <c r="E111" s="4"/>
-      <c r="F111" s="4"/>
-    </row>
-    <row r="112" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B111" s="3"/>
+      <c r="C111" s="3"/>
+      <c r="D111" s="3"/>
+      <c r="E111" s="3"/>
+      <c r="F111" s="3"/>
+    </row>
+    <row r="112" spans="1:6" ht="12.6" customHeight="1">
       <c r="A112" s="2"/>
-      <c r="B112" s="4"/>
-      <c r="C112" s="4"/>
-      <c r="D112" s="4"/>
-      <c r="E112" s="4"/>
-      <c r="F112" s="4"/>
-    </row>
-    <row r="113" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B112" s="3"/>
+      <c r="C112" s="3"/>
+      <c r="D112" s="3"/>
+      <c r="E112" s="3"/>
+      <c r="F112" s="3"/>
+    </row>
+    <row r="113" spans="1:6" ht="12.6" customHeight="1">
       <c r="A113" s="2"/>
-      <c r="B113" s="4"/>
-      <c r="C113" s="4"/>
-      <c r="D113" s="4"/>
-      <c r="E113" s="4"/>
-      <c r="F113" s="4"/>
-    </row>
-    <row r="114" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B113" s="3"/>
+      <c r="C113" s="3"/>
+      <c r="D113" s="3"/>
+      <c r="E113" s="3"/>
+      <c r="F113" s="3"/>
+    </row>
+    <row r="114" spans="1:6" ht="12.6" customHeight="1">
       <c r="A114" s="2"/>
-      <c r="B114" s="4"/>
-      <c r="C114" s="4"/>
-      <c r="D114" s="4"/>
-      <c r="E114" s="4"/>
-      <c r="F114" s="4"/>
-    </row>
-    <row r="115" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B114" s="3"/>
+      <c r="C114" s="3"/>
+      <c r="D114" s="3"/>
+      <c r="E114" s="3"/>
+      <c r="F114" s="3"/>
+    </row>
+    <row r="115" spans="1:6" ht="12.6" customHeight="1">
       <c r="A115" s="2"/>
-      <c r="B115" s="4"/>
-      <c r="C115" s="4"/>
-      <c r="D115" s="4"/>
-      <c r="E115" s="4"/>
-      <c r="F115" s="4"/>
-    </row>
-    <row r="116" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B115" s="3"/>
+      <c r="C115" s="3"/>
+      <c r="D115" s="3"/>
+      <c r="E115" s="3"/>
+      <c r="F115" s="3"/>
+    </row>
+    <row r="116" spans="1:6" ht="12.6" customHeight="1">
       <c r="A116" s="2"/>
-      <c r="B116" s="4"/>
-      <c r="C116" s="4"/>
-      <c r="D116" s="4"/>
-      <c r="E116" s="4"/>
-      <c r="F116" s="4"/>
-    </row>
-    <row r="117" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B116" s="3"/>
+      <c r="C116" s="3"/>
+      <c r="D116" s="3"/>
+      <c r="E116" s="3"/>
+      <c r="F116" s="3"/>
+    </row>
+    <row r="117" spans="1:6" ht="12.6" customHeight="1">
       <c r="A117" s="2"/>
-      <c r="B117" s="4"/>
-      <c r="C117" s="4"/>
-      <c r="D117" s="4"/>
-      <c r="E117" s="4"/>
-      <c r="F117" s="4"/>
-    </row>
-    <row r="118" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B117" s="3"/>
+      <c r="C117" s="3"/>
+      <c r="D117" s="3"/>
+      <c r="E117" s="3"/>
+      <c r="F117" s="3"/>
+    </row>
+    <row r="118" spans="1:6" ht="12.6" customHeight="1">
       <c r="A118" s="2"/>
-      <c r="B118" s="4"/>
-      <c r="C118" s="4"/>
-      <c r="D118" s="4"/>
-      <c r="E118" s="4"/>
-      <c r="F118" s="4"/>
-    </row>
-    <row r="119" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B118" s="3"/>
+      <c r="C118" s="3"/>
+      <c r="D118" s="3"/>
+      <c r="E118" s="3"/>
+      <c r="F118" s="3"/>
+    </row>
+    <row r="119" spans="1:6" ht="12.6" customHeight="1">
       <c r="A119" s="2"/>
-      <c r="B119" s="4"/>
-      <c r="C119" s="4"/>
-      <c r="D119" s="4"/>
-      <c r="E119" s="4"/>
-      <c r="F119" s="4"/>
-    </row>
-    <row r="120" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B119" s="3"/>
+      <c r="C119" s="3"/>
+      <c r="D119" s="3"/>
+      <c r="E119" s="3"/>
+      <c r="F119" s="3"/>
+    </row>
+    <row r="120" spans="1:6" ht="12.6" customHeight="1">
       <c r="A120" s="2"/>
-      <c r="B120" s="4"/>
-      <c r="C120" s="4"/>
-      <c r="D120" s="4"/>
-      <c r="E120" s="4"/>
-      <c r="F120" s="4"/>
-    </row>
-    <row r="121" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B120" s="3"/>
+      <c r="C120" s="3"/>
+      <c r="D120" s="3"/>
+      <c r="E120" s="3"/>
+      <c r="F120" s="3"/>
+    </row>
+    <row r="121" spans="1:6" ht="12.6" customHeight="1">
       <c r="A121" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>